<commit_message>
added 4x4, 8x8 draw line
</commit_message>
<xml_diff>
--- a/doc/hough created.xlsx
+++ b/doc/hough created.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kushn\projects\cv-workbench\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8248F74C-5C46-4BE5-AEAC-1E42BF5FEACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530C9309-0373-4241-9CAA-DE9CAB2748BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1416" yWindow="192" windowWidth="20508" windowHeight="11688" xr2:uid="{EEFBBBD4-DAC4-4F35-8600-CC9D3F6E2E33}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{EEFBBBD4-DAC4-4F35-8600-CC9D3F6E2E33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -429,7 +429,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -464,7 +464,8 @@
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -848,14 +849,6 @@
       </c>
     </row>
     <row r="6" spans="1:43" x14ac:dyDescent="0.3">
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="34"/>
-      <c r="Q6" s="34"/>
-      <c r="R6" s="34"/>
       <c r="W6" t="s">
         <v>1</v>
       </c>
@@ -894,7 +887,7 @@
         <v>-3.5</v>
       </c>
       <c r="H7">
-        <f t="shared" ref="H5:V7" si="0">H8-$X$6+0.5</f>
+        <f t="shared" ref="H7:V7" si="0">H8-$X$6+0.5</f>
         <v>-2.5</v>
       </c>
       <c r="I7">
@@ -1323,6 +1316,9 @@
         <f t="shared" si="6"/>
         <v>-0.45096523880948203</v>
       </c>
+      <c r="AJ11">
+        <v>0</v>
+      </c>
       <c r="AK11" s="18">
         <f>($AG$23-1)*(AB11-$AG$22)/$AG$20</f>
         <v>-1.9894280465094287E-5</v>
@@ -1433,6 +1429,9 @@
       <c r="AH12" s="28">
         <f t="shared" si="6"/>
         <v>-0.81698943430342108</v>
+      </c>
+      <c r="AJ12">
+        <v>1</v>
       </c>
       <c r="AK12" s="18">
         <f t="shared" ref="AK12:AK16" si="16">($AG$23-1)*(AB12-$AG$22)/$AG$20</f>
@@ -1537,6 +1536,9 @@
         <f t="shared" si="6"/>
         <v>-1.1830136297973599</v>
       </c>
+      <c r="AJ13">
+        <v>2</v>
+      </c>
       <c r="AK13" s="18">
         <f t="shared" si="16"/>
         <v>3.5999880634317218</v>
@@ -1637,6 +1639,9 @@
         <f t="shared" si="6"/>
         <v>-1.5490378252912991</v>
       </c>
+      <c r="AJ14">
+        <v>3</v>
+      </c>
       <c r="AK14" s="18">
         <f t="shared" si="16"/>
         <v>5.399992042287816</v>
@@ -1736,6 +1741,9 @@
       <c r="AH15" s="28">
         <f t="shared" si="6"/>
         <v>-1.9150620207852378</v>
+      </c>
+      <c r="AJ15">
+        <v>4</v>
       </c>
       <c r="AK15" s="18">
         <f t="shared" si="16"/>
@@ -1838,6 +1846,9 @@
         <f t="shared" si="6"/>
         <v>-2.281086216279177</v>
       </c>
+      <c r="AJ16">
+        <v>5</v>
+      </c>
       <c r="AK16" s="18">
         <f t="shared" si="16"/>
         <v>9</v>
@@ -1951,7 +1962,21 @@
       <c r="AK18">
         <v>1</v>
       </c>
-      <c r="AN18" s="33"/>
+      <c r="AL18">
+        <v>0</v>
+      </c>
+      <c r="AM18">
+        <v>0</v>
+      </c>
+      <c r="AN18" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO18">
+        <v>0</v>
+      </c>
+      <c r="AP18">
+        <v>0</v>
+      </c>
       <c r="AQ18">
         <v>1</v>
       </c>
@@ -2006,12 +2031,26 @@
       <c r="AJ19">
         <v>1</v>
       </c>
+      <c r="AK19">
+        <v>0</v>
+      </c>
       <c r="AL19">
         <v>1</v>
       </c>
-      <c r="AN19" s="33"/>
+      <c r="AM19">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO19">
+        <v>0</v>
+      </c>
       <c r="AP19">
         <v>1</v>
+      </c>
+      <c r="AQ19">
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:43" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2071,7 +2110,21 @@
       <c r="AK20">
         <v>1</v>
       </c>
-      <c r="AN20" s="33"/>
+      <c r="AL20">
+        <v>0</v>
+      </c>
+      <c r="AM20">
+        <v>0</v>
+      </c>
+      <c r="AN20" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO20">
+        <v>0</v>
+      </c>
+      <c r="AP20">
+        <v>0</v>
+      </c>
       <c r="AQ20">
         <v>1</v>
       </c>
@@ -2122,15 +2175,26 @@
       <c r="AJ21">
         <v>3</v>
       </c>
+      <c r="AK21">
+        <v>0</v>
+      </c>
       <c r="AL21">
         <v>1</v>
       </c>
       <c r="AM21">
         <v>2</v>
       </c>
-      <c r="AN21" s="33"/>
+      <c r="AN21" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO21">
+        <v>2</v>
+      </c>
       <c r="AP21">
         <v>1</v>
+      </c>
+      <c r="AQ21">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:43" x14ac:dyDescent="0.3">
@@ -2179,30 +2243,32 @@
         <f>MIN(AB12:AH17)</f>
         <v>-2.281086216279177</v>
       </c>
-      <c r="AI22" s="18">
+      <c r="AI22" s="32">
         <f t="shared" si="18"/>
         <v>-1.4676968855240493</v>
       </c>
-      <c r="AJ22">
+      <c r="AJ22" s="33">
         <v>4</v>
       </c>
-      <c r="AK22">
-        <v>1</v>
-      </c>
-      <c r="AL22">
-        <v>1</v>
-      </c>
-      <c r="AM22">
-        <v>1</v>
-      </c>
-      <c r="AN22" s="33"/>
-      <c r="AO22">
-        <v>2</v>
-      </c>
-      <c r="AP22">
-        <v>1</v>
-      </c>
-      <c r="AQ22">
+      <c r="AK22" s="33">
+        <v>1</v>
+      </c>
+      <c r="AL22" s="33">
+        <v>1</v>
+      </c>
+      <c r="AM22" s="33">
+        <v>1</v>
+      </c>
+      <c r="AN22" s="33">
+        <v>6</v>
+      </c>
+      <c r="AO22" s="33">
+        <v>1</v>
+      </c>
+      <c r="AP22" s="33">
+        <v>1</v>
+      </c>
+      <c r="AQ22" s="33">
         <v>1</v>
       </c>
     </row>
@@ -2251,32 +2317,32 @@
       <c r="AG23" s="29">
         <v>10</v>
       </c>
-      <c r="AI23" s="32">
+      <c r="AI23" s="34">
         <f t="shared" si="18"/>
         <v>-1.2643495528352675</v>
       </c>
-      <c r="AJ23" s="33">
+      <c r="AJ23" s="35">
         <v>5</v>
       </c>
-      <c r="AK23" s="33">
-        <v>1</v>
-      </c>
-      <c r="AL23" s="33">
-        <v>1</v>
-      </c>
-      <c r="AM23" s="33">
+      <c r="AK23">
+        <v>1</v>
+      </c>
+      <c r="AL23">
+        <v>1</v>
+      </c>
+      <c r="AM23">
         <v>2</v>
       </c>
       <c r="AN23" s="33">
-        <v>6</v>
-      </c>
-      <c r="AO23" s="33">
-        <v>1</v>
-      </c>
-      <c r="AP23" s="33">
-        <v>1</v>
-      </c>
-      <c r="AQ23" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO23">
+        <v>2</v>
+      </c>
+      <c r="AP23">
+        <v>1</v>
+      </c>
+      <c r="AQ23">
         <v>1</v>
       </c>
     </row>
@@ -2332,17 +2398,26 @@
       <c r="AJ24">
         <v>6</v>
       </c>
+      <c r="AK24">
+        <v>0</v>
+      </c>
       <c r="AL24">
         <v>1</v>
       </c>
       <c r="AM24">
         <v>1</v>
       </c>
+      <c r="AN24" s="33">
+        <v>0</v>
+      </c>
       <c r="AO24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AP24">
         <v>1</v>
+      </c>
+      <c r="AQ24">
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:43" x14ac:dyDescent="0.3">
@@ -2381,8 +2456,14 @@
       <c r="AL25">
         <v>1</v>
       </c>
+      <c r="AM25">
+        <v>0</v>
+      </c>
+      <c r="AN25" s="33">
+        <v>0</v>
+      </c>
       <c r="AO25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP25">
         <v>1</v>
@@ -2412,6 +2493,27 @@
       </c>
       <c r="AJ26">
         <v>8</v>
+      </c>
+      <c r="AK26">
+        <v>0</v>
+      </c>
+      <c r="AL26">
+        <v>0</v>
+      </c>
+      <c r="AM26">
+        <v>0</v>
+      </c>
+      <c r="AN26" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO26">
+        <v>0</v>
+      </c>
+      <c r="AP26">
+        <v>0</v>
+      </c>
+      <c r="AQ26">
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:43" x14ac:dyDescent="0.3">
@@ -2439,6 +2541,21 @@
       </c>
       <c r="AK27">
         <v>1</v>
+      </c>
+      <c r="AL27">
+        <v>0</v>
+      </c>
+      <c r="AM27">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="33">
+        <v>0</v>
+      </c>
+      <c r="AO27">
+        <v>0</v>
+      </c>
+      <c r="AP27">
+        <v>0</v>
       </c>
       <c r="AQ27">
         <v>1</v>

</xml_diff>